<commit_message>
Agregar evidencias del proyecto
</commit_message>
<xml_diff>
--- a/Cronograma/Itinerario-Ayo_Alisson V1.xlsx
+++ b/Cronograma/Itinerario-Ayo_Alisson V1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MSI\Desktop\Prácticas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MSI\Desktop\Prácticas\37009_PPP\Cronograma\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF2655FE-E6B1-49AC-A699-59D02DFE57A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D577DFF9-6C86-4F06-B1EF-BAA483C11488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ActividadesDetalle" sheetId="5" r:id="rId1"/>
@@ -860,10 +860,22 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" textRotation="255" wrapText="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
@@ -884,20 +896,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" textRotation="255" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1192,15 +1192,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="24" x14ac:dyDescent="0.7">
-      <c r="B1" s="35" t="s">
+      <c r="B1" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A2" s="4" t="s">
@@ -1268,10 +1268,10 @@
       </c>
     </row>
     <row r="9" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A9" s="32">
+      <c r="A9" s="23">
         <v>46279</v>
       </c>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="23" t="s">
         <v>18</v>
       </c>
       <c r="C9" s="14" t="s">
@@ -1281,17 +1281,17 @@
         <v>2</v>
       </c>
       <c r="E9" s="14"/>
-      <c r="F9" s="33" t="s">
+      <c r="F9" s="25" t="s">
         <v>170</v>
       </c>
-      <c r="G9" s="34">
-        <v>6</v>
-      </c>
-      <c r="H9" s="23"/>
+      <c r="G9" s="26">
+        <v>6</v>
+      </c>
+      <c r="H9" s="35"/>
     </row>
     <row r="10" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A10" s="32"/>
-      <c r="B10" s="32"/>
+      <c r="A10" s="23"/>
+      <c r="B10" s="23"/>
       <c r="C10" s="14" t="s">
         <v>20</v>
       </c>
@@ -1299,13 +1299,13 @@
         <v>2</v>
       </c>
       <c r="E10" s="14"/>
-      <c r="F10" s="33"/>
-      <c r="G10" s="34"/>
-      <c r="H10" s="23"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="26"/>
+      <c r="H10" s="35"/>
     </row>
     <row r="11" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A11" s="32"/>
-      <c r="B11" s="32"/>
+      <c r="A11" s="23"/>
+      <c r="B11" s="23"/>
       <c r="C11" s="14" t="s">
         <v>21</v>
       </c>
@@ -1316,15 +1316,15 @@
         <f>SUM(D9:D11)</f>
         <v>6</v>
       </c>
-      <c r="F11" s="33"/>
-      <c r="G11" s="34"/>
-      <c r="H11" s="23"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="35"/>
     </row>
     <row r="12" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A12" s="32">
+      <c r="A12" s="23">
         <v>46280</v>
       </c>
-      <c r="B12" s="32" t="s">
+      <c r="B12" s="23" t="s">
         <v>23</v>
       </c>
       <c r="C12" s="14" t="s">
@@ -1334,17 +1334,17 @@
         <v>2</v>
       </c>
       <c r="E12" s="14"/>
-      <c r="F12" s="33" t="s">
+      <c r="F12" s="25" t="s">
         <v>171</v>
       </c>
-      <c r="G12" s="34">
-        <v>6</v>
-      </c>
-      <c r="H12" s="23"/>
+      <c r="G12" s="26">
+        <v>6</v>
+      </c>
+      <c r="H12" s="35"/>
     </row>
     <row r="13" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A13" s="32"/>
-      <c r="B13" s="32"/>
+      <c r="A13" s="23"/>
+      <c r="B13" s="23"/>
       <c r="C13" s="14" t="s">
         <v>25</v>
       </c>
@@ -1352,13 +1352,13 @@
         <v>2</v>
       </c>
       <c r="E13" s="13"/>
-      <c r="F13" s="33"/>
-      <c r="G13" s="34"/>
-      <c r="H13" s="23"/>
+      <c r="F13" s="25"/>
+      <c r="G13" s="26"/>
+      <c r="H13" s="35"/>
     </row>
     <row r="14" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A14" s="32"/>
-      <c r="B14" s="32"/>
+      <c r="A14" s="23"/>
+      <c r="B14" s="23"/>
       <c r="C14" s="14" t="s">
         <v>22</v>
       </c>
@@ -1368,15 +1368,15 @@
       <c r="E14" s="14">
         <v>6</v>
       </c>
-      <c r="F14" s="33"/>
-      <c r="G14" s="34"/>
-      <c r="H14" s="23"/>
+      <c r="F14" s="25"/>
+      <c r="G14" s="26"/>
+      <c r="H14" s="35"/>
     </row>
     <row r="15" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A15" s="32">
+      <c r="A15" s="23">
         <v>46281</v>
       </c>
-      <c r="B15" s="32" t="s">
+      <c r="B15" s="23" t="s">
         <v>26</v>
       </c>
       <c r="C15" s="14" t="s">
@@ -1386,17 +1386,17 @@
         <v>2</v>
       </c>
       <c r="E15" s="13"/>
-      <c r="F15" s="33" t="s">
+      <c r="F15" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G15" s="34">
-        <v>6</v>
-      </c>
-      <c r="H15" s="23"/>
+      <c r="G15" s="26">
+        <v>6</v>
+      </c>
+      <c r="H15" s="35"/>
     </row>
     <row r="16" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A16" s="32"/>
-      <c r="B16" s="32"/>
+      <c r="A16" s="23"/>
+      <c r="B16" s="23"/>
       <c r="C16" s="21" t="s">
         <v>28</v>
       </c>
@@ -1404,13 +1404,13 @@
         <v>2</v>
       </c>
       <c r="E16" s="13"/>
-      <c r="F16" s="33"/>
-      <c r="G16" s="34"/>
-      <c r="H16" s="23"/>
+      <c r="F16" s="25"/>
+      <c r="G16" s="26"/>
+      <c r="H16" s="35"/>
     </row>
     <row r="17" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A17" s="32"/>
-      <c r="B17" s="32"/>
+      <c r="A17" s="23"/>
+      <c r="B17" s="23"/>
       <c r="C17" s="21" t="s">
         <v>29</v>
       </c>
@@ -1420,15 +1420,15 @@
       <c r="E17" s="14">
         <v>6</v>
       </c>
-      <c r="F17" s="33"/>
-      <c r="G17" s="34"/>
-      <c r="H17" s="23"/>
+      <c r="F17" s="25"/>
+      <c r="G17" s="26"/>
+      <c r="H17" s="35"/>
     </row>
     <row r="18" spans="1:8" ht="54" x14ac:dyDescent="0.5">
-      <c r="A18" s="32">
+      <c r="A18" s="23">
         <v>46282</v>
       </c>
-      <c r="B18" s="32" t="s">
+      <c r="B18" s="23" t="s">
         <v>30</v>
       </c>
       <c r="C18" s="14" t="s">
@@ -1438,17 +1438,17 @@
         <v>2</v>
       </c>
       <c r="E18" s="13"/>
-      <c r="F18" s="33" t="s">
+      <c r="F18" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G18" s="34">
-        <v>6</v>
-      </c>
-      <c r="H18" s="23"/>
+      <c r="G18" s="26">
+        <v>6</v>
+      </c>
+      <c r="H18" s="35"/>
     </row>
     <row r="19" spans="1:8" ht="38.4" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A19" s="32"/>
-      <c r="B19" s="32"/>
+      <c r="A19" s="23"/>
+      <c r="B19" s="23"/>
       <c r="C19" s="14" t="s">
         <v>32</v>
       </c>
@@ -1456,13 +1456,13 @@
         <v>2</v>
       </c>
       <c r="E19" s="13"/>
-      <c r="F19" s="33"/>
-      <c r="G19" s="34"/>
-      <c r="H19" s="23"/>
+      <c r="F19" s="25"/>
+      <c r="G19" s="26"/>
+      <c r="H19" s="35"/>
     </row>
     <row r="20" spans="1:8" ht="54" x14ac:dyDescent="0.5">
-      <c r="A20" s="32"/>
-      <c r="B20" s="32"/>
+      <c r="A20" s="23"/>
+      <c r="B20" s="23"/>
       <c r="C20" s="14" t="s">
         <v>33</v>
       </c>
@@ -1472,15 +1472,15 @@
       <c r="E20" s="14">
         <v>6</v>
       </c>
-      <c r="F20" s="33"/>
-      <c r="G20" s="34"/>
-      <c r="H20" s="23"/>
+      <c r="F20" s="25"/>
+      <c r="G20" s="26"/>
+      <c r="H20" s="35"/>
     </row>
     <row r="21" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A21" s="32">
+      <c r="A21" s="23">
         <v>46283</v>
       </c>
-      <c r="B21" s="32" t="s">
+      <c r="B21" s="23" t="s">
         <v>34</v>
       </c>
       <c r="C21" s="14" t="s">
@@ -1490,17 +1490,17 @@
         <v>2</v>
       </c>
       <c r="E21" s="13"/>
-      <c r="F21" s="33" t="s">
+      <c r="F21" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G21" s="34">
-        <v>6</v>
-      </c>
-      <c r="H21" s="23"/>
+      <c r="G21" s="26">
+        <v>6</v>
+      </c>
+      <c r="H21" s="35"/>
     </row>
     <row r="22" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A22" s="32"/>
-      <c r="B22" s="32"/>
+      <c r="A22" s="23"/>
+      <c r="B22" s="23"/>
       <c r="C22" s="14" t="s">
         <v>36</v>
       </c>
@@ -1508,13 +1508,13 @@
         <v>2</v>
       </c>
       <c r="E22" s="13"/>
-      <c r="F22" s="33"/>
-      <c r="G22" s="34"/>
-      <c r="H22" s="23"/>
+      <c r="F22" s="25"/>
+      <c r="G22" s="26"/>
+      <c r="H22" s="35"/>
     </row>
     <row r="23" spans="1:8" ht="54" x14ac:dyDescent="0.5">
-      <c r="A23" s="32"/>
-      <c r="B23" s="32"/>
+      <c r="A23" s="23"/>
+      <c r="B23" s="23"/>
       <c r="C23" s="14" t="s">
         <v>37</v>
       </c>
@@ -1524,15 +1524,15 @@
       <c r="E23" s="14">
         <v>6</v>
       </c>
-      <c r="F23" s="33"/>
-      <c r="G23" s="34"/>
-      <c r="H23" s="23"/>
+      <c r="F23" s="25"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="35"/>
     </row>
     <row r="24" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A24" s="32">
+      <c r="A24" s="23">
         <v>46286</v>
       </c>
-      <c r="B24" s="32" t="s">
+      <c r="B24" s="23" t="s">
         <v>38</v>
       </c>
       <c r="C24" s="14" t="s">
@@ -1542,17 +1542,17 @@
         <v>2</v>
       </c>
       <c r="E24" s="14"/>
-      <c r="F24" s="33" t="s">
+      <c r="F24" s="25" t="s">
         <v>171</v>
       </c>
-      <c r="G24" s="34">
-        <v>6</v>
-      </c>
-      <c r="H24" s="23"/>
+      <c r="G24" s="26">
+        <v>6</v>
+      </c>
+      <c r="H24" s="35"/>
     </row>
     <row r="25" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A25" s="32"/>
-      <c r="B25" s="32"/>
+      <c r="A25" s="23"/>
+      <c r="B25" s="23"/>
       <c r="C25" s="14" t="s">
         <v>40</v>
       </c>
@@ -1560,13 +1560,13 @@
         <v>2</v>
       </c>
       <c r="E25" s="13"/>
-      <c r="F25" s="33"/>
-      <c r="G25" s="34"/>
-      <c r="H25" s="23"/>
+      <c r="F25" s="25"/>
+      <c r="G25" s="26"/>
+      <c r="H25" s="35"/>
     </row>
     <row r="26" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A26" s="32"/>
-      <c r="B26" s="32"/>
+      <c r="A26" s="23"/>
+      <c r="B26" s="23"/>
       <c r="C26" s="14" t="s">
         <v>41</v>
       </c>
@@ -1576,15 +1576,15 @@
       <c r="E26" s="14">
         <v>6</v>
       </c>
-      <c r="F26" s="33"/>
-      <c r="G26" s="34"/>
-      <c r="H26" s="23"/>
+      <c r="F26" s="25"/>
+      <c r="G26" s="26"/>
+      <c r="H26" s="35"/>
     </row>
     <row r="27" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A27" s="32">
+      <c r="A27" s="23">
         <v>46287</v>
       </c>
-      <c r="B27" s="32" t="s">
+      <c r="B27" s="23" t="s">
         <v>42</v>
       </c>
       <c r="C27" s="14" t="s">
@@ -1594,17 +1594,17 @@
         <v>2</v>
       </c>
       <c r="E27" s="13"/>
-      <c r="F27" s="33" t="s">
+      <c r="F27" s="25" t="s">
         <v>171</v>
       </c>
-      <c r="G27" s="34">
-        <v>6</v>
-      </c>
-      <c r="H27" s="23"/>
+      <c r="G27" s="26">
+        <v>6</v>
+      </c>
+      <c r="H27" s="35"/>
     </row>
     <row r="28" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A28" s="32"/>
-      <c r="B28" s="32"/>
+      <c r="A28" s="23"/>
+      <c r="B28" s="23"/>
       <c r="C28" s="14" t="s">
         <v>44</v>
       </c>
@@ -1612,13 +1612,13 @@
         <v>2</v>
       </c>
       <c r="E28" s="13"/>
-      <c r="F28" s="33"/>
-      <c r="G28" s="34"/>
-      <c r="H28" s="23"/>
+      <c r="F28" s="25"/>
+      <c r="G28" s="26"/>
+      <c r="H28" s="35"/>
     </row>
     <row r="29" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A29" s="32"/>
-      <c r="B29" s="32"/>
+      <c r="A29" s="23"/>
+      <c r="B29" s="23"/>
       <c r="C29" s="14" t="s">
         <v>45</v>
       </c>
@@ -1628,15 +1628,15 @@
       <c r="E29" s="14">
         <v>6</v>
       </c>
-      <c r="F29" s="33"/>
-      <c r="G29" s="34"/>
-      <c r="H29" s="23"/>
+      <c r="F29" s="25"/>
+      <c r="G29" s="26"/>
+      <c r="H29" s="35"/>
     </row>
     <row r="30" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A30" s="32">
+      <c r="A30" s="23">
         <v>46288</v>
       </c>
-      <c r="B30" s="32" t="s">
+      <c r="B30" s="23" t="s">
         <v>46</v>
       </c>
       <c r="C30" s="14" t="s">
@@ -1646,17 +1646,17 @@
         <v>2</v>
       </c>
       <c r="E30" s="13"/>
-      <c r="F30" s="33" t="s">
+      <c r="F30" s="25" t="s">
         <v>171</v>
       </c>
-      <c r="G30" s="34">
-        <v>6</v>
-      </c>
-      <c r="H30" s="23"/>
+      <c r="G30" s="26">
+        <v>6</v>
+      </c>
+      <c r="H30" s="35"/>
     </row>
     <row r="31" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A31" s="32"/>
-      <c r="B31" s="32"/>
+      <c r="A31" s="23"/>
+      <c r="B31" s="23"/>
       <c r="C31" s="14" t="s">
         <v>48</v>
       </c>
@@ -1664,13 +1664,13 @@
         <v>2</v>
       </c>
       <c r="E31" s="13"/>
-      <c r="F31" s="33"/>
-      <c r="G31" s="34"/>
-      <c r="H31" s="23"/>
+      <c r="F31" s="25"/>
+      <c r="G31" s="26"/>
+      <c r="H31" s="35"/>
     </row>
     <row r="32" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A32" s="32"/>
-      <c r="B32" s="32"/>
+      <c r="A32" s="23"/>
+      <c r="B32" s="23"/>
       <c r="C32" s="14" t="s">
         <v>49</v>
       </c>
@@ -1680,15 +1680,15 @@
       <c r="E32" s="14">
         <v>6</v>
       </c>
-      <c r="F32" s="33"/>
-      <c r="G32" s="34"/>
-      <c r="H32" s="23"/>
+      <c r="F32" s="25"/>
+      <c r="G32" s="26"/>
+      <c r="H32" s="35"/>
     </row>
     <row r="33" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A33" s="32">
+      <c r="A33" s="23">
         <v>46289</v>
       </c>
-      <c r="B33" s="32" t="s">
+      <c r="B33" s="23" t="s">
         <v>50</v>
       </c>
       <c r="C33" s="14" t="s">
@@ -1698,17 +1698,17 @@
         <v>2</v>
       </c>
       <c r="E33" s="13"/>
-      <c r="F33" s="33" t="s">
+      <c r="F33" s="25" t="s">
         <v>171</v>
       </c>
-      <c r="G33" s="34">
-        <v>6</v>
-      </c>
-      <c r="H33" s="23"/>
+      <c r="G33" s="26">
+        <v>6</v>
+      </c>
+      <c r="H33" s="35"/>
     </row>
     <row r="34" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A34" s="32"/>
-      <c r="B34" s="32"/>
+      <c r="A34" s="23"/>
+      <c r="B34" s="23"/>
       <c r="C34" s="14" t="s">
         <v>52</v>
       </c>
@@ -1716,13 +1716,13 @@
         <v>2</v>
       </c>
       <c r="E34" s="13"/>
-      <c r="F34" s="33"/>
-      <c r="G34" s="34"/>
-      <c r="H34" s="23"/>
+      <c r="F34" s="25"/>
+      <c r="G34" s="26"/>
+      <c r="H34" s="35"/>
     </row>
     <row r="35" spans="1:8" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A35" s="32"/>
-      <c r="B35" s="32"/>
+      <c r="A35" s="23"/>
+      <c r="B35" s="23"/>
       <c r="C35" s="14" t="s">
         <v>53</v>
       </c>
@@ -1732,15 +1732,15 @@
       <c r="E35" s="14">
         <v>6</v>
       </c>
-      <c r="F35" s="33"/>
-      <c r="G35" s="34"/>
-      <c r="H35" s="23"/>
+      <c r="F35" s="25"/>
+      <c r="G35" s="26"/>
+      <c r="H35" s="35"/>
     </row>
     <row r="36" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A36" s="32">
+      <c r="A36" s="23">
         <v>46290</v>
       </c>
-      <c r="B36" s="32" t="s">
+      <c r="B36" s="23" t="s">
         <v>17</v>
       </c>
       <c r="C36" s="14" t="s">
@@ -1750,17 +1750,17 @@
         <v>2</v>
       </c>
       <c r="E36" s="14"/>
-      <c r="F36" s="33" t="s">
+      <c r="F36" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G36" s="34">
-        <v>6</v>
-      </c>
-      <c r="H36" s="23"/>
+      <c r="G36" s="26">
+        <v>6</v>
+      </c>
+      <c r="H36" s="35"/>
     </row>
     <row r="37" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A37" s="32"/>
-      <c r="B37" s="32"/>
+      <c r="A37" s="23"/>
+      <c r="B37" s="23"/>
       <c r="C37" s="14" t="s">
         <v>55</v>
       </c>
@@ -1768,13 +1768,13 @@
         <v>2</v>
       </c>
       <c r="E37" s="13"/>
-      <c r="F37" s="33"/>
-      <c r="G37" s="34"/>
-      <c r="H37" s="23"/>
+      <c r="F37" s="25"/>
+      <c r="G37" s="26"/>
+      <c r="H37" s="35"/>
     </row>
     <row r="38" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A38" s="32"/>
-      <c r="B38" s="32"/>
+      <c r="A38" s="23"/>
+      <c r="B38" s="23"/>
       <c r="C38" s="14" t="s">
         <v>56</v>
       </c>
@@ -1784,15 +1784,15 @@
       <c r="E38" s="14">
         <v>6</v>
       </c>
-      <c r="F38" s="33"/>
-      <c r="G38" s="34"/>
-      <c r="H38" s="23"/>
+      <c r="F38" s="25"/>
+      <c r="G38" s="26"/>
+      <c r="H38" s="35"/>
     </row>
     <row r="39" spans="1:8" ht="25.8" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A39" s="32">
+      <c r="A39" s="23">
         <v>46293</v>
       </c>
-      <c r="B39" s="32" t="s">
+      <c r="B39" s="23" t="s">
         <v>57</v>
       </c>
       <c r="C39" s="14" t="s">
@@ -1802,17 +1802,17 @@
         <v>2</v>
       </c>
       <c r="E39" s="13"/>
-      <c r="F39" s="33" t="s">
+      <c r="F39" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G39" s="34">
-        <v>6</v>
-      </c>
-      <c r="H39" s="23"/>
+      <c r="G39" s="26">
+        <v>6</v>
+      </c>
+      <c r="H39" s="35"/>
     </row>
     <row r="40" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A40" s="32"/>
-      <c r="B40" s="32"/>
+      <c r="A40" s="23"/>
+      <c r="B40" s="23"/>
       <c r="C40" s="14" t="s">
         <v>59</v>
       </c>
@@ -1820,13 +1820,13 @@
         <v>2</v>
       </c>
       <c r="E40" s="13"/>
-      <c r="F40" s="33"/>
-      <c r="G40" s="34"/>
-      <c r="H40" s="23"/>
+      <c r="F40" s="25"/>
+      <c r="G40" s="26"/>
+      <c r="H40" s="35"/>
     </row>
     <row r="41" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A41" s="32"/>
-      <c r="B41" s="32"/>
+      <c r="A41" s="23"/>
+      <c r="B41" s="23"/>
       <c r="C41" s="14" t="s">
         <v>60</v>
       </c>
@@ -1836,15 +1836,15 @@
       <c r="E41" s="14">
         <v>6</v>
       </c>
-      <c r="F41" s="33"/>
-      <c r="G41" s="34"/>
-      <c r="H41" s="23"/>
+      <c r="F41" s="25"/>
+      <c r="G41" s="26"/>
+      <c r="H41" s="35"/>
     </row>
     <row r="42" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A42" s="32">
+      <c r="A42" s="23">
         <v>46294</v>
       </c>
-      <c r="B42" s="32" t="s">
+      <c r="B42" s="23" t="s">
         <v>61</v>
       </c>
       <c r="C42" s="14" t="s">
@@ -1854,17 +1854,17 @@
         <v>2</v>
       </c>
       <c r="E42" s="13"/>
-      <c r="F42" s="33" t="s">
+      <c r="F42" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G42" s="34">
-        <v>6</v>
-      </c>
-      <c r="H42" s="23"/>
+      <c r="G42" s="26">
+        <v>6</v>
+      </c>
+      <c r="H42" s="35"/>
     </row>
     <row r="43" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A43" s="32"/>
-      <c r="B43" s="32"/>
+      <c r="A43" s="23"/>
+      <c r="B43" s="23"/>
       <c r="C43" s="14" t="s">
         <v>63</v>
       </c>
@@ -1872,13 +1872,13 @@
         <v>2</v>
       </c>
       <c r="E43" s="13"/>
-      <c r="F43" s="33"/>
-      <c r="G43" s="34"/>
-      <c r="H43" s="23"/>
+      <c r="F43" s="25"/>
+      <c r="G43" s="26"/>
+      <c r="H43" s="35"/>
     </row>
     <row r="44" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A44" s="32"/>
-      <c r="B44" s="32"/>
+      <c r="A44" s="23"/>
+      <c r="B44" s="23"/>
       <c r="C44" s="14" t="s">
         <v>64</v>
       </c>
@@ -1888,15 +1888,15 @@
       <c r="E44" s="14">
         <v>6</v>
       </c>
-      <c r="F44" s="33"/>
-      <c r="G44" s="34"/>
-      <c r="H44" s="23"/>
+      <c r="F44" s="25"/>
+      <c r="G44" s="26"/>
+      <c r="H44" s="35"/>
     </row>
     <row r="45" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A45" s="32">
+      <c r="A45" s="23">
         <v>46295</v>
       </c>
-      <c r="B45" s="32" t="s">
+      <c r="B45" s="23" t="s">
         <v>65</v>
       </c>
       <c r="C45" s="14" t="s">
@@ -1906,17 +1906,17 @@
         <v>2</v>
       </c>
       <c r="E45" s="13"/>
-      <c r="F45" s="33" t="s">
+      <c r="F45" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G45" s="34">
-        <v>6</v>
-      </c>
-      <c r="H45" s="23"/>
+      <c r="G45" s="26">
+        <v>6</v>
+      </c>
+      <c r="H45" s="35"/>
     </row>
     <row r="46" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A46" s="32"/>
-      <c r="B46" s="32"/>
+      <c r="A46" s="23"/>
+      <c r="B46" s="23"/>
       <c r="C46" s="14" t="s">
         <v>67</v>
       </c>
@@ -1924,13 +1924,13 @@
         <v>2</v>
       </c>
       <c r="E46" s="13"/>
-      <c r="F46" s="33"/>
-      <c r="G46" s="34"/>
-      <c r="H46" s="23"/>
+      <c r="F46" s="25"/>
+      <c r="G46" s="26"/>
+      <c r="H46" s="35"/>
     </row>
     <row r="47" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A47" s="32"/>
-      <c r="B47" s="32"/>
+      <c r="A47" s="23"/>
+      <c r="B47" s="23"/>
       <c r="C47" s="14" t="s">
         <v>68</v>
       </c>
@@ -1940,15 +1940,15 @@
       <c r="E47" s="14">
         <v>6</v>
       </c>
-      <c r="F47" s="33"/>
-      <c r="G47" s="34"/>
-      <c r="H47" s="23"/>
+      <c r="F47" s="25"/>
+      <c r="G47" s="26"/>
+      <c r="H47" s="35"/>
     </row>
     <row r="48" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A48" s="32">
+      <c r="A48" s="23">
         <v>46296</v>
       </c>
-      <c r="B48" s="32" t="s">
+      <c r="B48" s="23" t="s">
         <v>69</v>
       </c>
       <c r="C48" s="14" t="s">
@@ -1958,17 +1958,17 @@
         <v>2</v>
       </c>
       <c r="E48" s="13"/>
-      <c r="F48" s="33" t="s">
+      <c r="F48" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G48" s="34">
-        <v>6</v>
-      </c>
-      <c r="H48" s="23"/>
+      <c r="G48" s="26">
+        <v>6</v>
+      </c>
+      <c r="H48" s="35"/>
     </row>
     <row r="49" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A49" s="32"/>
-      <c r="B49" s="32"/>
+      <c r="A49" s="23"/>
+      <c r="B49" s="23"/>
       <c r="C49" s="14" t="s">
         <v>71</v>
       </c>
@@ -1976,13 +1976,13 @@
         <v>2</v>
       </c>
       <c r="E49" s="13"/>
-      <c r="F49" s="33"/>
-      <c r="G49" s="34"/>
-      <c r="H49" s="23"/>
+      <c r="F49" s="25"/>
+      <c r="G49" s="26"/>
+      <c r="H49" s="35"/>
     </row>
     <row r="50" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A50" s="32"/>
-      <c r="B50" s="32"/>
+      <c r="A50" s="23"/>
+      <c r="B50" s="23"/>
       <c r="C50" s="14" t="s">
         <v>72</v>
       </c>
@@ -1992,15 +1992,15 @@
       <c r="E50" s="14">
         <v>6</v>
       </c>
-      <c r="F50" s="33"/>
-      <c r="G50" s="34"/>
-      <c r="H50" s="23"/>
+      <c r="F50" s="25"/>
+      <c r="G50" s="26"/>
+      <c r="H50" s="35"/>
     </row>
     <row r="51" spans="1:8" ht="27.6" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A51" s="32">
+      <c r="A51" s="23">
         <v>46297</v>
       </c>
-      <c r="B51" s="32" t="s">
+      <c r="B51" s="23" t="s">
         <v>73</v>
       </c>
       <c r="C51" s="14" t="s">
@@ -2010,17 +2010,17 @@
         <v>2</v>
       </c>
       <c r="E51" s="13"/>
-      <c r="F51" s="33" t="s">
+      <c r="F51" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G51" s="34">
-        <v>6</v>
-      </c>
-      <c r="H51" s="23"/>
+      <c r="G51" s="26">
+        <v>6</v>
+      </c>
+      <c r="H51" s="35"/>
     </row>
     <row r="52" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A52" s="32"/>
-      <c r="B52" s="32"/>
+      <c r="A52" s="23"/>
+      <c r="B52" s="23"/>
       <c r="C52" s="14" t="s">
         <v>75</v>
       </c>
@@ -2028,13 +2028,13 @@
         <v>2</v>
       </c>
       <c r="E52" s="13"/>
-      <c r="F52" s="33"/>
-      <c r="G52" s="34"/>
-      <c r="H52" s="23"/>
+      <c r="F52" s="25"/>
+      <c r="G52" s="26"/>
+      <c r="H52" s="35"/>
     </row>
     <row r="53" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A53" s="32"/>
-      <c r="B53" s="32"/>
+      <c r="A53" s="23"/>
+      <c r="B53" s="23"/>
       <c r="C53" s="14" t="s">
         <v>76</v>
       </c>
@@ -2044,15 +2044,15 @@
       <c r="E53" s="14">
         <v>6</v>
       </c>
-      <c r="F53" s="33"/>
-      <c r="G53" s="34"/>
-      <c r="H53" s="23"/>
+      <c r="F53" s="25"/>
+      <c r="G53" s="26"/>
+      <c r="H53" s="35"/>
     </row>
     <row r="54" spans="1:8" ht="30.6" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A54" s="32">
+      <c r="A54" s="23">
         <v>46300</v>
       </c>
-      <c r="B54" s="32" t="s">
+      <c r="B54" s="23" t="s">
         <v>77</v>
       </c>
       <c r="C54" s="14" t="s">
@@ -2062,17 +2062,17 @@
         <v>2</v>
       </c>
       <c r="E54" s="13"/>
-      <c r="F54" s="33" t="s">
+      <c r="F54" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G54" s="34">
-        <v>6</v>
-      </c>
-      <c r="H54" s="23"/>
+      <c r="G54" s="26">
+        <v>6</v>
+      </c>
+      <c r="H54" s="35"/>
     </row>
     <row r="55" spans="1:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A55" s="32"/>
-      <c r="B55" s="32"/>
+      <c r="A55" s="23"/>
+      <c r="B55" s="23"/>
       <c r="C55" s="14" t="s">
         <v>79</v>
       </c>
@@ -2080,13 +2080,13 @@
         <v>2</v>
       </c>
       <c r="E55" s="13"/>
-      <c r="F55" s="33"/>
-      <c r="G55" s="34"/>
-      <c r="H55" s="23"/>
+      <c r="F55" s="25"/>
+      <c r="G55" s="26"/>
+      <c r="H55" s="35"/>
     </row>
     <row r="56" spans="1:8" ht="27.6" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A56" s="32"/>
-      <c r="B56" s="32"/>
+      <c r="A56" s="23"/>
+      <c r="B56" s="23"/>
       <c r="C56" s="14" t="s">
         <v>80</v>
       </c>
@@ -2096,15 +2096,15 @@
       <c r="E56" s="14">
         <v>6</v>
       </c>
-      <c r="F56" s="33"/>
-      <c r="G56" s="34"/>
-      <c r="H56" s="23"/>
+      <c r="F56" s="25"/>
+      <c r="G56" s="26"/>
+      <c r="H56" s="35"/>
     </row>
     <row r="57" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A57" s="32">
+      <c r="A57" s="23">
         <v>46301</v>
       </c>
-      <c r="B57" s="32" t="s">
+      <c r="B57" s="23" t="s">
         <v>81</v>
       </c>
       <c r="C57" s="14" t="s">
@@ -2114,17 +2114,17 @@
         <v>2</v>
       </c>
       <c r="E57" s="13"/>
-      <c r="F57" s="33" t="s">
+      <c r="F57" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G57" s="34">
-        <v>6</v>
-      </c>
-      <c r="H57" s="23"/>
+      <c r="G57" s="26">
+        <v>6</v>
+      </c>
+      <c r="H57" s="35"/>
     </row>
     <row r="58" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A58" s="32"/>
-      <c r="B58" s="32"/>
+      <c r="A58" s="23"/>
+      <c r="B58" s="23"/>
       <c r="C58" s="14" t="s">
         <v>83</v>
       </c>
@@ -2132,13 +2132,13 @@
         <v>2</v>
       </c>
       <c r="E58" s="13"/>
-      <c r="F58" s="33"/>
-      <c r="G58" s="34"/>
-      <c r="H58" s="23"/>
+      <c r="F58" s="25"/>
+      <c r="G58" s="26"/>
+      <c r="H58" s="35"/>
     </row>
     <row r="59" spans="1:8" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A59" s="32"/>
-      <c r="B59" s="32"/>
+      <c r="A59" s="23"/>
+      <c r="B59" s="23"/>
       <c r="C59" s="14" t="s">
         <v>84</v>
       </c>
@@ -2148,15 +2148,15 @@
       <c r="E59" s="14">
         <v>6</v>
       </c>
-      <c r="F59" s="33"/>
-      <c r="G59" s="34"/>
-      <c r="H59" s="23"/>
+      <c r="F59" s="25"/>
+      <c r="G59" s="26"/>
+      <c r="H59" s="35"/>
     </row>
     <row r="60" spans="1:8" ht="28.2" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A60" s="32">
+      <c r="A60" s="23">
         <v>46302</v>
       </c>
-      <c r="B60" s="32" t="s">
+      <c r="B60" s="23" t="s">
         <v>85</v>
       </c>
       <c r="C60" s="14" t="s">
@@ -2166,17 +2166,17 @@
         <v>2</v>
       </c>
       <c r="E60" s="13"/>
-      <c r="F60" s="33" t="s">
+      <c r="F60" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G60" s="34">
-        <v>6</v>
-      </c>
-      <c r="H60" s="23"/>
+      <c r="G60" s="26">
+        <v>6</v>
+      </c>
+      <c r="H60" s="35"/>
     </row>
     <row r="61" spans="1:8" ht="25.8" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A61" s="32"/>
-      <c r="B61" s="32"/>
+      <c r="A61" s="23"/>
+      <c r="B61" s="23"/>
       <c r="C61" s="14" t="s">
         <v>87</v>
       </c>
@@ -2184,13 +2184,13 @@
         <v>2</v>
       </c>
       <c r="E61" s="13"/>
-      <c r="F61" s="33"/>
-      <c r="G61" s="34"/>
-      <c r="H61" s="23"/>
+      <c r="F61" s="25"/>
+      <c r="G61" s="26"/>
+      <c r="H61" s="35"/>
     </row>
     <row r="62" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A62" s="32"/>
-      <c r="B62" s="32"/>
+      <c r="A62" s="23"/>
+      <c r="B62" s="23"/>
       <c r="C62" s="14" t="s">
         <v>88</v>
       </c>
@@ -2200,15 +2200,15 @@
       <c r="E62" s="14">
         <v>6</v>
       </c>
-      <c r="F62" s="33"/>
-      <c r="G62" s="34"/>
-      <c r="H62" s="23"/>
+      <c r="F62" s="25"/>
+      <c r="G62" s="26"/>
+      <c r="H62" s="35"/>
     </row>
     <row r="63" spans="1:8" ht="31.8" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A63" s="32">
+      <c r="A63" s="23">
         <v>46303</v>
       </c>
-      <c r="B63" s="32" t="s">
+      <c r="B63" s="23" t="s">
         <v>89</v>
       </c>
       <c r="C63" s="14" t="s">
@@ -2218,17 +2218,17 @@
         <v>2</v>
       </c>
       <c r="E63" s="13"/>
-      <c r="F63" s="33" t="s">
+      <c r="F63" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G63" s="34">
-        <v>6</v>
-      </c>
-      <c r="H63" s="23"/>
+      <c r="G63" s="26">
+        <v>6</v>
+      </c>
+      <c r="H63" s="35"/>
     </row>
     <row r="64" spans="1:8" ht="24.6" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A64" s="32"/>
-      <c r="B64" s="32"/>
+      <c r="A64" s="23"/>
+      <c r="B64" s="23"/>
       <c r="C64" s="14" t="s">
         <v>91</v>
       </c>
@@ -2236,13 +2236,13 @@
         <v>2</v>
       </c>
       <c r="E64" s="13"/>
-      <c r="F64" s="33"/>
-      <c r="G64" s="34"/>
-      <c r="H64" s="23"/>
+      <c r="F64" s="25"/>
+      <c r="G64" s="26"/>
+      <c r="H64" s="35"/>
     </row>
     <row r="65" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A65" s="32"/>
-      <c r="B65" s="32"/>
+      <c r="A65" s="23"/>
+      <c r="B65" s="23"/>
       <c r="C65" s="14" t="s">
         <v>92</v>
       </c>
@@ -2252,15 +2252,15 @@
       <c r="E65" s="14">
         <v>6</v>
       </c>
-      <c r="F65" s="33"/>
-      <c r="G65" s="34"/>
-      <c r="H65" s="23"/>
+      <c r="F65" s="25"/>
+      <c r="G65" s="26"/>
+      <c r="H65" s="35"/>
     </row>
     <row r="66" spans="1:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A66" s="32">
+      <c r="A66" s="23">
         <v>46307</v>
       </c>
-      <c r="B66" s="32" t="s">
+      <c r="B66" s="23" t="s">
         <v>93</v>
       </c>
       <c r="C66" s="14" t="s">
@@ -2270,17 +2270,17 @@
         <v>2</v>
       </c>
       <c r="E66" s="13"/>
-      <c r="F66" s="33" t="s">
+      <c r="F66" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G66" s="34">
-        <v>6</v>
-      </c>
-      <c r="H66" s="23"/>
+      <c r="G66" s="26">
+        <v>6</v>
+      </c>
+      <c r="H66" s="35"/>
     </row>
     <row r="67" spans="1:8" ht="32.4" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A67" s="32"/>
-      <c r="B67" s="32"/>
+      <c r="A67" s="23"/>
+      <c r="B67" s="23"/>
       <c r="C67" s="14" t="s">
         <v>95</v>
       </c>
@@ -2288,13 +2288,13 @@
         <v>2</v>
       </c>
       <c r="E67" s="14"/>
-      <c r="F67" s="33"/>
-      <c r="G67" s="34"/>
-      <c r="H67" s="23"/>
+      <c r="F67" s="25"/>
+      <c r="G67" s="26"/>
+      <c r="H67" s="35"/>
     </row>
     <row r="68" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A68" s="32"/>
-      <c r="B68" s="32"/>
+      <c r="A68" s="23"/>
+      <c r="B68" s="23"/>
       <c r="C68" s="14" t="s">
         <v>96</v>
       </c>
@@ -2304,15 +2304,15 @@
       <c r="E68" s="14">
         <v>6</v>
       </c>
-      <c r="F68" s="33"/>
-      <c r="G68" s="34"/>
-      <c r="H68" s="23"/>
+      <c r="F68" s="25"/>
+      <c r="G68" s="26"/>
+      <c r="H68" s="35"/>
     </row>
     <row r="69" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A69" s="32">
+      <c r="A69" s="23">
         <v>46308</v>
       </c>
-      <c r="B69" s="34" t="s">
+      <c r="B69" s="26" t="s">
         <v>97</v>
       </c>
       <c r="C69" s="14" t="s">
@@ -2322,17 +2322,17 @@
         <v>2</v>
       </c>
       <c r="E69" s="14"/>
-      <c r="F69" s="33" t="s">
+      <c r="F69" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G69" s="34">
-        <v>6</v>
-      </c>
-      <c r="H69" s="23"/>
+      <c r="G69" s="26">
+        <v>6</v>
+      </c>
+      <c r="H69" s="35"/>
     </row>
     <row r="70" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A70" s="32"/>
-      <c r="B70" s="34"/>
+      <c r="A70" s="23"/>
+      <c r="B70" s="26"/>
       <c r="C70" s="14" t="s">
         <v>99</v>
       </c>
@@ -2340,13 +2340,13 @@
         <v>2</v>
       </c>
       <c r="E70" s="14"/>
-      <c r="F70" s="33"/>
-      <c r="G70" s="34"/>
-      <c r="H70" s="23"/>
+      <c r="F70" s="25"/>
+      <c r="G70" s="26"/>
+      <c r="H70" s="35"/>
     </row>
     <row r="71" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A71" s="32"/>
-      <c r="B71" s="34"/>
+      <c r="A71" s="23"/>
+      <c r="B71" s="26"/>
       <c r="C71" s="14" t="s">
         <v>100</v>
       </c>
@@ -2356,15 +2356,15 @@
       <c r="E71" s="14">
         <v>6</v>
       </c>
-      <c r="F71" s="33"/>
-      <c r="G71" s="34"/>
-      <c r="H71" s="23"/>
+      <c r="F71" s="25"/>
+      <c r="G71" s="26"/>
+      <c r="H71" s="35"/>
     </row>
     <row r="72" spans="1:8" ht="31.8" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A72" s="32">
+      <c r="A72" s="23">
         <v>46309</v>
       </c>
-      <c r="B72" s="34" t="s">
+      <c r="B72" s="26" t="s">
         <v>101</v>
       </c>
       <c r="C72" s="14" t="s">
@@ -2374,17 +2374,17 @@
         <v>2</v>
       </c>
       <c r="E72" s="14"/>
-      <c r="F72" s="33" t="s">
+      <c r="F72" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G72" s="34">
-        <v>6</v>
-      </c>
-      <c r="H72" s="23"/>
+      <c r="G72" s="26">
+        <v>6</v>
+      </c>
+      <c r="H72" s="35"/>
     </row>
     <row r="73" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A73" s="32"/>
-      <c r="B73" s="34"/>
+      <c r="A73" s="23"/>
+      <c r="B73" s="26"/>
       <c r="C73" s="14" t="s">
         <v>103</v>
       </c>
@@ -2392,13 +2392,13 @@
         <v>2</v>
       </c>
       <c r="E73" s="14"/>
-      <c r="F73" s="33"/>
-      <c r="G73" s="34"/>
-      <c r="H73" s="23"/>
+      <c r="F73" s="25"/>
+      <c r="G73" s="26"/>
+      <c r="H73" s="35"/>
     </row>
     <row r="74" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A74" s="32"/>
-      <c r="B74" s="34"/>
+      <c r="A74" s="23"/>
+      <c r="B74" s="26"/>
       <c r="C74" s="14" t="s">
         <v>104</v>
       </c>
@@ -2408,15 +2408,15 @@
       <c r="E74" s="14">
         <v>6</v>
       </c>
-      <c r="F74" s="33"/>
-      <c r="G74" s="34"/>
-      <c r="H74" s="23"/>
+      <c r="F74" s="25"/>
+      <c r="G74" s="26"/>
+      <c r="H74" s="35"/>
     </row>
     <row r="75" spans="1:8" ht="25.8" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A75" s="32">
+      <c r="A75" s="23">
         <v>46310</v>
       </c>
-      <c r="B75" s="34" t="s">
+      <c r="B75" s="26" t="s">
         <v>105</v>
       </c>
       <c r="C75" s="14" t="s">
@@ -2426,17 +2426,17 @@
         <v>2</v>
       </c>
       <c r="E75" s="14"/>
-      <c r="F75" s="33" t="s">
+      <c r="F75" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G75" s="34">
-        <v>6</v>
-      </c>
-      <c r="H75" s="23"/>
+      <c r="G75" s="26">
+        <v>6</v>
+      </c>
+      <c r="H75" s="35"/>
     </row>
     <row r="76" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A76" s="32"/>
-      <c r="B76" s="34"/>
+      <c r="A76" s="23"/>
+      <c r="B76" s="26"/>
       <c r="C76" s="14" t="s">
         <v>107</v>
       </c>
@@ -2444,13 +2444,13 @@
         <v>2</v>
       </c>
       <c r="E76" s="14"/>
-      <c r="F76" s="33"/>
-      <c r="G76" s="34"/>
-      <c r="H76" s="23"/>
+      <c r="F76" s="25"/>
+      <c r="G76" s="26"/>
+      <c r="H76" s="35"/>
     </row>
     <row r="77" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A77" s="32"/>
-      <c r="B77" s="34"/>
+      <c r="A77" s="23"/>
+      <c r="B77" s="26"/>
       <c r="C77" s="14" t="s">
         <v>108</v>
       </c>
@@ -2460,15 +2460,15 @@
       <c r="E77" s="14">
         <v>6</v>
       </c>
-      <c r="F77" s="33"/>
-      <c r="G77" s="34"/>
-      <c r="H77" s="23"/>
+      <c r="F77" s="25"/>
+      <c r="G77" s="26"/>
+      <c r="H77" s="35"/>
     </row>
     <row r="78" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A78" s="32">
+      <c r="A78" s="23">
         <v>46311</v>
       </c>
-      <c r="B78" s="32" t="s">
+      <c r="B78" s="23" t="s">
         <v>109</v>
       </c>
       <c r="C78" s="14" t="s">
@@ -2478,17 +2478,17 @@
         <v>2</v>
       </c>
       <c r="E78" s="14"/>
-      <c r="F78" s="33" t="s">
+      <c r="F78" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G78" s="34">
-        <v>6</v>
-      </c>
-      <c r="H78" s="23"/>
+      <c r="G78" s="26">
+        <v>6</v>
+      </c>
+      <c r="H78" s="35"/>
     </row>
     <row r="79" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A79" s="32"/>
-      <c r="B79" s="32"/>
+      <c r="A79" s="23"/>
+      <c r="B79" s="23"/>
       <c r="C79" s="14" t="s">
         <v>111</v>
       </c>
@@ -2496,13 +2496,13 @@
         <v>2</v>
       </c>
       <c r="E79" s="14"/>
-      <c r="F79" s="33"/>
-      <c r="G79" s="34"/>
-      <c r="H79" s="23"/>
+      <c r="F79" s="25"/>
+      <c r="G79" s="26"/>
+      <c r="H79" s="35"/>
     </row>
     <row r="80" spans="1:8" ht="33.6" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A80" s="32"/>
-      <c r="B80" s="32"/>
+      <c r="A80" s="23"/>
+      <c r="B80" s="23"/>
       <c r="C80" s="14" t="s">
         <v>112</v>
       </c>
@@ -2512,15 +2512,15 @@
       <c r="E80" s="14">
         <v>6</v>
       </c>
-      <c r="F80" s="33"/>
-      <c r="G80" s="34"/>
-      <c r="H80" s="23"/>
+      <c r="F80" s="25"/>
+      <c r="G80" s="26"/>
+      <c r="H80" s="35"/>
     </row>
     <row r="81" spans="1:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A81" s="31">
+      <c r="A81" s="27">
         <v>46314</v>
       </c>
-      <c r="B81" s="32" t="s">
+      <c r="B81" s="23" t="s">
         <v>109</v>
       </c>
       <c r="C81" s="21" t="s">
@@ -2530,17 +2530,17 @@
         <v>3</v>
       </c>
       <c r="E81" s="14"/>
-      <c r="F81" s="33" t="s">
+      <c r="F81" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G81" s="34">
+      <c r="G81" s="26">
         <v>6</v>
       </c>
       <c r="H81" s="24"/>
     </row>
     <row r="82" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A82" s="31"/>
-      <c r="B82" s="32"/>
+      <c r="A82" s="27"/>
+      <c r="B82" s="23"/>
       <c r="C82" s="14" t="s">
         <v>114</v>
       </c>
@@ -2550,15 +2550,15 @@
       <c r="E82" s="14">
         <v>6</v>
       </c>
-      <c r="F82" s="33"/>
-      <c r="G82" s="34"/>
+      <c r="F82" s="25"/>
+      <c r="G82" s="26"/>
       <c r="H82" s="24"/>
     </row>
     <row r="83" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A83" s="31">
+      <c r="A83" s="27">
         <v>46315</v>
       </c>
-      <c r="B83" s="32" t="s">
+      <c r="B83" s="23" t="s">
         <v>109</v>
       </c>
       <c r="C83" s="14" t="s">
@@ -2568,17 +2568,17 @@
         <v>3</v>
       </c>
       <c r="E83" s="14"/>
-      <c r="F83" s="33" t="s">
+      <c r="F83" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G83" s="34">
-        <v>6</v>
-      </c>
-      <c r="H83" s="23"/>
+      <c r="G83" s="26">
+        <v>6</v>
+      </c>
+      <c r="H83" s="35"/>
     </row>
     <row r="84" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A84" s="31"/>
-      <c r="B84" s="32"/>
+      <c r="A84" s="27"/>
+      <c r="B84" s="23"/>
       <c r="C84" s="21" t="s">
         <v>116</v>
       </c>
@@ -2588,15 +2588,15 @@
       <c r="E84" s="14">
         <v>6</v>
       </c>
-      <c r="F84" s="33"/>
-      <c r="G84" s="34"/>
-      <c r="H84" s="23"/>
+      <c r="F84" s="25"/>
+      <c r="G84" s="26"/>
+      <c r="H84" s="35"/>
     </row>
     <row r="85" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A85" s="32">
+      <c r="A85" s="23">
         <v>46316</v>
       </c>
-      <c r="B85" s="32" t="s">
+      <c r="B85" s="23" t="s">
         <v>117</v>
       </c>
       <c r="C85" s="14" t="s">
@@ -2606,17 +2606,17 @@
         <v>2</v>
       </c>
       <c r="E85" s="14"/>
-      <c r="F85" s="33" t="s">
+      <c r="F85" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G85" s="34">
-        <v>6</v>
-      </c>
-      <c r="H85" s="23"/>
+      <c r="G85" s="26">
+        <v>6</v>
+      </c>
+      <c r="H85" s="35"/>
     </row>
     <row r="86" spans="1:8" ht="24.6" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A86" s="32"/>
-      <c r="B86" s="32"/>
+      <c r="A86" s="23"/>
+      <c r="B86" s="23"/>
       <c r="C86" s="14" t="s">
         <v>119</v>
       </c>
@@ -2624,13 +2624,13 @@
         <v>2</v>
       </c>
       <c r="E86" s="13"/>
-      <c r="F86" s="33"/>
-      <c r="G86" s="34"/>
-      <c r="H86" s="23"/>
+      <c r="F86" s="25"/>
+      <c r="G86" s="26"/>
+      <c r="H86" s="35"/>
     </row>
     <row r="87" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A87" s="32"/>
-      <c r="B87" s="32"/>
+      <c r="A87" s="23"/>
+      <c r="B87" s="23"/>
       <c r="C87" s="14" t="s">
         <v>120</v>
       </c>
@@ -2640,15 +2640,15 @@
       <c r="E87" s="14">
         <v>6</v>
       </c>
-      <c r="F87" s="33"/>
-      <c r="G87" s="34"/>
-      <c r="H87" s="23"/>
+      <c r="F87" s="25"/>
+      <c r="G87" s="26"/>
+      <c r="H87" s="35"/>
     </row>
     <row r="88" spans="1:8" ht="27.6" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A88" s="32">
+      <c r="A88" s="23">
         <v>46317</v>
       </c>
-      <c r="B88" s="34" t="s">
+      <c r="B88" s="26" t="s">
         <v>117</v>
       </c>
       <c r="C88" s="14" t="s">
@@ -2658,17 +2658,17 @@
         <v>3</v>
       </c>
       <c r="E88" s="13"/>
-      <c r="F88" s="33" t="s">
+      <c r="F88" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G88" s="34">
-        <v>6</v>
-      </c>
-      <c r="H88" s="23"/>
+      <c r="G88" s="26">
+        <v>6</v>
+      </c>
+      <c r="H88" s="35"/>
     </row>
     <row r="89" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A89" s="32"/>
-      <c r="B89" s="34"/>
+      <c r="A89" s="23"/>
+      <c r="B89" s="26"/>
       <c r="C89" s="14" t="s">
         <v>122</v>
       </c>
@@ -2678,15 +2678,15 @@
       <c r="E89" s="14">
         <v>6</v>
       </c>
-      <c r="F89" s="33"/>
-      <c r="G89" s="34"/>
-      <c r="H89" s="23"/>
+      <c r="F89" s="25"/>
+      <c r="G89" s="26"/>
+      <c r="H89" s="35"/>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A90" s="32">
+      <c r="A90" s="23">
         <v>46318</v>
       </c>
-      <c r="B90" s="34" t="s">
+      <c r="B90" s="26" t="s">
         <v>117</v>
       </c>
       <c r="C90" s="21" t="s">
@@ -2696,17 +2696,17 @@
         <v>3</v>
       </c>
       <c r="E90" s="13"/>
-      <c r="F90" s="33" t="s">
+      <c r="F90" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G90" s="34">
-        <v>6</v>
-      </c>
-      <c r="H90" s="23"/>
+      <c r="G90" s="26">
+        <v>6</v>
+      </c>
+      <c r="H90" s="35"/>
     </row>
     <row r="91" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A91" s="32"/>
-      <c r="B91" s="34"/>
+      <c r="A91" s="23"/>
+      <c r="B91" s="26"/>
       <c r="C91" s="14" t="s">
         <v>124</v>
       </c>
@@ -2716,15 +2716,15 @@
       <c r="E91" s="14">
         <v>6</v>
       </c>
-      <c r="F91" s="33"/>
-      <c r="G91" s="34"/>
-      <c r="H91" s="23"/>
+      <c r="F91" s="25"/>
+      <c r="G91" s="26"/>
+      <c r="H91" s="35"/>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A92" s="32">
+      <c r="A92" s="23">
         <v>46321</v>
       </c>
-      <c r="B92" s="34" t="s">
+      <c r="B92" s="26" t="s">
         <v>125</v>
       </c>
       <c r="C92" s="14" t="s">
@@ -2734,17 +2734,17 @@
         <v>2</v>
       </c>
       <c r="E92" s="14"/>
-      <c r="F92" s="33" t="s">
+      <c r="F92" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G92" s="34">
-        <v>6</v>
-      </c>
-      <c r="H92" s="23"/>
+      <c r="G92" s="26">
+        <v>6</v>
+      </c>
+      <c r="H92" s="35"/>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A93" s="32"/>
-      <c r="B93" s="34"/>
+      <c r="A93" s="23"/>
+      <c r="B93" s="26"/>
       <c r="C93" s="20" t="s">
         <v>127</v>
       </c>
@@ -2752,13 +2752,13 @@
         <v>2</v>
       </c>
       <c r="E93" s="13"/>
-      <c r="F93" s="33"/>
-      <c r="G93" s="34"/>
-      <c r="H93" s="23"/>
+      <c r="F93" s="25"/>
+      <c r="G93" s="26"/>
+      <c r="H93" s="35"/>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A94" s="32"/>
-      <c r="B94" s="34"/>
+      <c r="A94" s="23"/>
+      <c r="B94" s="26"/>
       <c r="C94" s="14" t="s">
         <v>128</v>
       </c>
@@ -2768,15 +2768,15 @@
       <c r="E94" s="14">
         <v>6</v>
       </c>
-      <c r="F94" s="33"/>
-      <c r="G94" s="34"/>
-      <c r="H94" s="23"/>
+      <c r="F94" s="25"/>
+      <c r="G94" s="26"/>
+      <c r="H94" s="35"/>
     </row>
     <row r="95" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A95" s="32">
+      <c r="A95" s="23">
         <v>46322</v>
       </c>
-      <c r="B95" s="34" t="s">
+      <c r="B95" s="26" t="s">
         <v>125</v>
       </c>
       <c r="C95" s="14" t="s">
@@ -2786,17 +2786,17 @@
         <v>2</v>
       </c>
       <c r="E95" s="13"/>
-      <c r="F95" s="33" t="s">
+      <c r="F95" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G95" s="34">
-        <v>6</v>
-      </c>
-      <c r="H95" s="23"/>
+      <c r="G95" s="26">
+        <v>6</v>
+      </c>
+      <c r="H95" s="35"/>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A96" s="32"/>
-      <c r="B96" s="34"/>
+      <c r="A96" s="23"/>
+      <c r="B96" s="26"/>
       <c r="C96" s="14" t="s">
         <v>130</v>
       </c>
@@ -2804,13 +2804,13 @@
         <v>2</v>
       </c>
       <c r="E96" s="13"/>
-      <c r="F96" s="33"/>
-      <c r="G96" s="34"/>
-      <c r="H96" s="23"/>
+      <c r="F96" s="25"/>
+      <c r="G96" s="26"/>
+      <c r="H96" s="35"/>
     </row>
     <row r="97" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A97" s="32"/>
-      <c r="B97" s="34"/>
+      <c r="A97" s="23"/>
+      <c r="B97" s="26"/>
       <c r="C97" s="14" t="s">
         <v>131</v>
       </c>
@@ -2820,12 +2820,12 @@
       <c r="E97" s="14">
         <v>6</v>
       </c>
-      <c r="F97" s="33"/>
-      <c r="G97" s="34"/>
-      <c r="H97" s="23"/>
+      <c r="F97" s="25"/>
+      <c r="G97" s="26"/>
+      <c r="H97" s="35"/>
     </row>
     <row r="98" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A98" s="32">
+      <c r="A98" s="23">
         <v>46323</v>
       </c>
       <c r="B98" s="24" t="s">
@@ -2838,16 +2838,16 @@
         <v>2</v>
       </c>
       <c r="E98" s="14"/>
-      <c r="F98" s="33" t="s">
+      <c r="F98" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G98" s="34">
-        <v>6</v>
-      </c>
-      <c r="H98" s="23"/>
+      <c r="G98" s="26">
+        <v>6</v>
+      </c>
+      <c r="H98" s="35"/>
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A99" s="32"/>
+      <c r="A99" s="23"/>
       <c r="B99" s="24"/>
       <c r="C99" s="20" t="s">
         <v>134</v>
@@ -2856,12 +2856,12 @@
         <v>2</v>
       </c>
       <c r="E99" s="13"/>
-      <c r="F99" s="33"/>
-      <c r="G99" s="34"/>
-      <c r="H99" s="23"/>
+      <c r="F99" s="25"/>
+      <c r="G99" s="26"/>
+      <c r="H99" s="35"/>
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A100" s="32"/>
+      <c r="A100" s="23"/>
       <c r="B100" s="24"/>
       <c r="C100" s="14" t="s">
         <v>135</v>
@@ -2872,15 +2872,15 @@
       <c r="E100" s="14">
         <v>6</v>
       </c>
-      <c r="F100" s="33"/>
-      <c r="G100" s="34"/>
-      <c r="H100" s="23"/>
+      <c r="F100" s="25"/>
+      <c r="G100" s="26"/>
+      <c r="H100" s="35"/>
     </row>
     <row r="101" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A101" s="31">
+      <c r="A101" s="27">
         <v>46324</v>
       </c>
-      <c r="B101" s="33" t="s">
+      <c r="B101" s="25" t="s">
         <v>136</v>
       </c>
       <c r="C101" s="14" t="s">
@@ -2890,17 +2890,17 @@
         <v>2</v>
       </c>
       <c r="E101" s="13"/>
-      <c r="F101" s="33" t="s">
+      <c r="F101" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G101" s="34">
-        <v>6</v>
-      </c>
-      <c r="H101" s="23"/>
+      <c r="G101" s="26">
+        <v>6</v>
+      </c>
+      <c r="H101" s="35"/>
     </row>
     <row r="102" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A102" s="31"/>
-      <c r="B102" s="33"/>
+      <c r="A102" s="27"/>
+      <c r="B102" s="25"/>
       <c r="C102" s="14" t="s">
         <v>138</v>
       </c>
@@ -2908,13 +2908,13 @@
         <v>2</v>
       </c>
       <c r="E102" s="13"/>
-      <c r="F102" s="33"/>
-      <c r="G102" s="34"/>
-      <c r="H102" s="23"/>
+      <c r="F102" s="25"/>
+      <c r="G102" s="26"/>
+      <c r="H102" s="35"/>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A103" s="31"/>
-      <c r="B103" s="33"/>
+      <c r="A103" s="27"/>
+      <c r="B103" s="25"/>
       <c r="C103" s="14" t="s">
         <v>139</v>
       </c>
@@ -2924,15 +2924,15 @@
       <c r="E103" s="14">
         <v>6</v>
       </c>
-      <c r="F103" s="33"/>
-      <c r="G103" s="34"/>
-      <c r="H103" s="23"/>
+      <c r="F103" s="25"/>
+      <c r="G103" s="26"/>
+      <c r="H103" s="35"/>
     </row>
     <row r="104" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A104" s="32">
+      <c r="A104" s="23">
         <v>46325</v>
       </c>
-      <c r="B104" s="33" t="s">
+      <c r="B104" s="25" t="s">
         <v>140</v>
       </c>
       <c r="C104" s="14" t="s">
@@ -2942,17 +2942,17 @@
         <v>2</v>
       </c>
       <c r="E104" s="13"/>
-      <c r="F104" s="33" t="s">
+      <c r="F104" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G104" s="34">
-        <v>6</v>
-      </c>
-      <c r="H104" s="23"/>
+      <c r="G104" s="26">
+        <v>6</v>
+      </c>
+      <c r="H104" s="35"/>
     </row>
     <row r="105" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A105" s="32"/>
-      <c r="B105" s="33"/>
+      <c r="A105" s="23"/>
+      <c r="B105" s="25"/>
       <c r="C105" s="15" t="s">
         <v>142</v>
       </c>
@@ -2960,13 +2960,13 @@
         <v>2</v>
       </c>
       <c r="E105" s="13"/>
-      <c r="F105" s="33"/>
-      <c r="G105" s="34"/>
-      <c r="H105" s="23"/>
+      <c r="F105" s="25"/>
+      <c r="G105" s="26"/>
+      <c r="H105" s="35"/>
     </row>
     <row r="106" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A106" s="32"/>
-      <c r="B106" s="33"/>
+      <c r="A106" s="23"/>
+      <c r="B106" s="25"/>
       <c r="C106" s="14" t="s">
         <v>143</v>
       </c>
@@ -2976,15 +2976,15 @@
       <c r="E106" s="14">
         <v>6</v>
       </c>
-      <c r="F106" s="33"/>
-      <c r="G106" s="34"/>
-      <c r="H106" s="23"/>
+      <c r="F106" s="25"/>
+      <c r="G106" s="26"/>
+      <c r="H106" s="35"/>
     </row>
     <row r="107" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A107" s="32">
+      <c r="A107" s="23">
         <v>46330</v>
       </c>
-      <c r="B107" s="33" t="s">
+      <c r="B107" s="25" t="s">
         <v>144</v>
       </c>
       <c r="C107" s="14" t="s">
@@ -2994,17 +2994,17 @@
         <v>2</v>
       </c>
       <c r="E107" s="13"/>
-      <c r="F107" s="33" t="s">
+      <c r="F107" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G107" s="34">
-        <v>6</v>
-      </c>
-      <c r="H107" s="23"/>
+      <c r="G107" s="26">
+        <v>6</v>
+      </c>
+      <c r="H107" s="35"/>
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A108" s="32"/>
-      <c r="B108" s="33"/>
+      <c r="A108" s="23"/>
+      <c r="B108" s="25"/>
       <c r="C108" s="14" t="s">
         <v>147</v>
       </c>
@@ -3012,13 +3012,13 @@
         <v>2</v>
       </c>
       <c r="E108" s="13"/>
-      <c r="F108" s="33"/>
-      <c r="G108" s="34"/>
-      <c r="H108" s="23"/>
+      <c r="F108" s="25"/>
+      <c r="G108" s="26"/>
+      <c r="H108" s="35"/>
     </row>
     <row r="109" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A109" s="32"/>
-      <c r="B109" s="33"/>
+      <c r="A109" s="23"/>
+      <c r="B109" s="25"/>
       <c r="C109" s="14" t="s">
         <v>146</v>
       </c>
@@ -3028,15 +3028,15 @@
       <c r="E109" s="14">
         <v>6</v>
       </c>
-      <c r="F109" s="33"/>
-      <c r="G109" s="34"/>
-      <c r="H109" s="23"/>
+      <c r="F109" s="25"/>
+      <c r="G109" s="26"/>
+      <c r="H109" s="35"/>
     </row>
     <row r="110" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A110" s="32">
+      <c r="A110" s="23">
         <v>46331</v>
       </c>
-      <c r="B110" s="33" t="s">
+      <c r="B110" s="25" t="s">
         <v>148</v>
       </c>
       <c r="C110" s="14" t="s">
@@ -3046,17 +3046,17 @@
         <v>2</v>
       </c>
       <c r="E110" s="13"/>
-      <c r="F110" s="33" t="s">
+      <c r="F110" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G110" s="34">
-        <v>6</v>
-      </c>
-      <c r="H110" s="23"/>
+      <c r="G110" s="26">
+        <v>6</v>
+      </c>
+      <c r="H110" s="35"/>
     </row>
     <row r="111" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A111" s="32"/>
-      <c r="B111" s="33"/>
+      <c r="A111" s="23"/>
+      <c r="B111" s="25"/>
       <c r="C111" s="14" t="s">
         <v>150</v>
       </c>
@@ -3064,13 +3064,13 @@
         <v>2</v>
       </c>
       <c r="E111" s="13"/>
-      <c r="F111" s="33"/>
-      <c r="G111" s="34"/>
-      <c r="H111" s="23"/>
+      <c r="F111" s="25"/>
+      <c r="G111" s="26"/>
+      <c r="H111" s="35"/>
     </row>
     <row r="112" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A112" s="32"/>
-      <c r="B112" s="33"/>
+      <c r="A112" s="23"/>
+      <c r="B112" s="25"/>
       <c r="C112" s="14" t="s">
         <v>151</v>
       </c>
@@ -3080,15 +3080,15 @@
       <c r="E112" s="14">
         <v>6</v>
       </c>
-      <c r="F112" s="33"/>
-      <c r="G112" s="34"/>
-      <c r="H112" s="23"/>
+      <c r="F112" s="25"/>
+      <c r="G112" s="26"/>
+      <c r="H112" s="35"/>
     </row>
     <row r="113" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A113" s="32">
+      <c r="A113" s="23">
         <v>46332</v>
       </c>
-      <c r="B113" s="33" t="s">
+      <c r="B113" s="25" t="s">
         <v>152</v>
       </c>
       <c r="C113" s="14" t="s">
@@ -3098,17 +3098,17 @@
         <v>2</v>
       </c>
       <c r="E113" s="13"/>
-      <c r="F113" s="33" t="s">
+      <c r="F113" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G113" s="34">
-        <v>6</v>
-      </c>
-      <c r="H113" s="23"/>
+      <c r="G113" s="26">
+        <v>6</v>
+      </c>
+      <c r="H113" s="35"/>
     </row>
     <row r="114" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A114" s="32"/>
-      <c r="B114" s="33"/>
+      <c r="A114" s="23"/>
+      <c r="B114" s="25"/>
       <c r="C114" s="14" t="s">
         <v>154</v>
       </c>
@@ -3116,13 +3116,13 @@
         <v>2</v>
       </c>
       <c r="E114" s="13"/>
-      <c r="F114" s="33"/>
-      <c r="G114" s="34"/>
-      <c r="H114" s="23"/>
+      <c r="F114" s="25"/>
+      <c r="G114" s="26"/>
+      <c r="H114" s="35"/>
     </row>
     <row r="115" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A115" s="32"/>
-      <c r="B115" s="33"/>
+      <c r="A115" s="23"/>
+      <c r="B115" s="25"/>
       <c r="C115" s="14" t="s">
         <v>155</v>
       </c>
@@ -3132,59 +3132,59 @@
       <c r="E115" s="14">
         <v>6</v>
       </c>
-      <c r="F115" s="33"/>
-      <c r="G115" s="34"/>
-      <c r="H115" s="23"/>
+      <c r="F115" s="25"/>
+      <c r="G115" s="26"/>
+      <c r="H115" s="35"/>
     </row>
     <row r="116" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A116" s="32">
+      <c r="A116" s="23">
         <v>46335</v>
       </c>
-      <c r="B116" s="33" t="s">
+      <c r="B116" s="25" t="s">
         <v>167</v>
       </c>
-      <c r="C116" s="25" t="s">
+      <c r="C116" s="29" t="s">
         <v>168</v>
       </c>
-      <c r="D116" s="28">
-        <v>6</v>
-      </c>
-      <c r="E116" s="28">
-        <v>6</v>
-      </c>
-      <c r="F116" s="33" t="s">
+      <c r="D116" s="32">
+        <v>6</v>
+      </c>
+      <c r="E116" s="32">
+        <v>6</v>
+      </c>
+      <c r="F116" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G116" s="34">
-        <v>6</v>
-      </c>
-      <c r="H116" s="23"/>
+      <c r="G116" s="26">
+        <v>6</v>
+      </c>
+      <c r="H116" s="35"/>
     </row>
     <row r="117" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A117" s="32"/>
-      <c r="B117" s="33"/>
-      <c r="C117" s="26"/>
-      <c r="D117" s="29"/>
-      <c r="E117" s="29"/>
-      <c r="F117" s="33"/>
-      <c r="G117" s="34"/>
-      <c r="H117" s="23"/>
+      <c r="A117" s="23"/>
+      <c r="B117" s="25"/>
+      <c r="C117" s="30"/>
+      <c r="D117" s="33"/>
+      <c r="E117" s="33"/>
+      <c r="F117" s="25"/>
+      <c r="G117" s="26"/>
+      <c r="H117" s="35"/>
     </row>
     <row r="118" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A118" s="32"/>
-      <c r="B118" s="33"/>
-      <c r="C118" s="27"/>
-      <c r="D118" s="30"/>
-      <c r="E118" s="30"/>
-      <c r="F118" s="33"/>
-      <c r="G118" s="34"/>
-      <c r="H118" s="23"/>
+      <c r="A118" s="23"/>
+      <c r="B118" s="25"/>
+      <c r="C118" s="31"/>
+      <c r="D118" s="34"/>
+      <c r="E118" s="34"/>
+      <c r="F118" s="25"/>
+      <c r="G118" s="26"/>
+      <c r="H118" s="35"/>
     </row>
     <row r="119" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A119" s="32">
+      <c r="A119" s="23">
         <v>46336</v>
       </c>
-      <c r="B119" s="33" t="s">
+      <c r="B119" s="25" t="s">
         <v>156</v>
       </c>
       <c r="C119" s="14" t="s">
@@ -3194,17 +3194,17 @@
         <v>2</v>
       </c>
       <c r="E119" s="13"/>
-      <c r="F119" s="33" t="s">
+      <c r="F119" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G119" s="34">
-        <v>6</v>
-      </c>
-      <c r="H119" s="23"/>
+      <c r="G119" s="26">
+        <v>6</v>
+      </c>
+      <c r="H119" s="35"/>
     </row>
     <row r="120" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A120" s="32"/>
-      <c r="B120" s="33"/>
+      <c r="A120" s="23"/>
+      <c r="B120" s="25"/>
       <c r="C120" s="14" t="s">
         <v>158</v>
       </c>
@@ -3212,13 +3212,13 @@
         <v>2</v>
       </c>
       <c r="E120" s="13"/>
-      <c r="F120" s="33"/>
-      <c r="G120" s="34"/>
-      <c r="H120" s="23"/>
+      <c r="F120" s="25"/>
+      <c r="G120" s="26"/>
+      <c r="H120" s="35"/>
     </row>
     <row r="121" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A121" s="32"/>
-      <c r="B121" s="33"/>
+      <c r="A121" s="23"/>
+      <c r="B121" s="25"/>
       <c r="C121" s="14" t="s">
         <v>159</v>
       </c>
@@ -3228,15 +3228,15 @@
       <c r="E121" s="14">
         <v>6</v>
       </c>
-      <c r="F121" s="33"/>
-      <c r="G121" s="34"/>
-      <c r="H121" s="23"/>
+      <c r="F121" s="25"/>
+      <c r="G121" s="26"/>
+      <c r="H121" s="35"/>
     </row>
     <row r="122" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A122" s="32">
+      <c r="A122" s="23">
         <v>46337</v>
       </c>
-      <c r="B122" s="33" t="s">
+      <c r="B122" s="25" t="s">
         <v>160</v>
       </c>
       <c r="C122" s="14" t="s">
@@ -3246,17 +3246,17 @@
         <v>2</v>
       </c>
       <c r="E122" s="13"/>
-      <c r="F122" s="33" t="s">
+      <c r="F122" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="G122" s="34">
-        <v>6</v>
-      </c>
-      <c r="H122" s="23"/>
+      <c r="G122" s="26">
+        <v>6</v>
+      </c>
+      <c r="H122" s="35"/>
     </row>
     <row r="123" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A123" s="32"/>
-      <c r="B123" s="33"/>
+      <c r="A123" s="23"/>
+      <c r="B123" s="25"/>
       <c r="C123" s="14" t="s">
         <v>162</v>
       </c>
@@ -3264,13 +3264,13 @@
         <v>2</v>
       </c>
       <c r="E123" s="13"/>
-      <c r="F123" s="33"/>
-      <c r="G123" s="34"/>
-      <c r="H123" s="23"/>
+      <c r="F123" s="25"/>
+      <c r="G123" s="26"/>
+      <c r="H123" s="35"/>
     </row>
     <row r="124" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A124" s="32"/>
-      <c r="B124" s="33"/>
+      <c r="A124" s="23"/>
+      <c r="B124" s="25"/>
       <c r="C124" s="14" t="s">
         <v>163</v>
       </c>
@@ -3280,9 +3280,9 @@
       <c r="E124" s="14">
         <v>6</v>
       </c>
-      <c r="F124" s="33"/>
-      <c r="G124" s="34"/>
-      <c r="H124" s="23"/>
+      <c r="F124" s="25"/>
+      <c r="G124" s="26"/>
+      <c r="H124" s="35"/>
     </row>
     <row r="125" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A125" s="11"/>
@@ -3388,6 +3388,186 @@
     </row>
   </sheetData>
   <mergeCells count="204">
+    <mergeCell ref="H122:H124"/>
+    <mergeCell ref="H95:H97"/>
+    <mergeCell ref="H98:H100"/>
+    <mergeCell ref="H101:H103"/>
+    <mergeCell ref="H104:H106"/>
+    <mergeCell ref="H107:H109"/>
+    <mergeCell ref="H110:H112"/>
+    <mergeCell ref="H113:H115"/>
+    <mergeCell ref="H116:H118"/>
+    <mergeCell ref="H119:H121"/>
+    <mergeCell ref="H72:H74"/>
+    <mergeCell ref="H75:H77"/>
+    <mergeCell ref="H78:H80"/>
+    <mergeCell ref="H83:H84"/>
+    <mergeCell ref="H81:H82"/>
+    <mergeCell ref="H85:H87"/>
+    <mergeCell ref="H88:H89"/>
+    <mergeCell ref="H90:H91"/>
+    <mergeCell ref="H92:H94"/>
+    <mergeCell ref="C116:C118"/>
+    <mergeCell ref="D116:D118"/>
+    <mergeCell ref="E116:E118"/>
+    <mergeCell ref="H9:H11"/>
+    <mergeCell ref="H12:H14"/>
+    <mergeCell ref="H15:H17"/>
+    <mergeCell ref="H18:H20"/>
+    <mergeCell ref="H21:H23"/>
+    <mergeCell ref="H24:H26"/>
+    <mergeCell ref="H27:H29"/>
+    <mergeCell ref="H30:H32"/>
+    <mergeCell ref="H33:H35"/>
+    <mergeCell ref="H36:H38"/>
+    <mergeCell ref="H39:H41"/>
+    <mergeCell ref="H42:H44"/>
+    <mergeCell ref="H45:H47"/>
+    <mergeCell ref="H48:H50"/>
+    <mergeCell ref="H51:H53"/>
+    <mergeCell ref="H54:H56"/>
+    <mergeCell ref="H57:H59"/>
+    <mergeCell ref="H60:H62"/>
+    <mergeCell ref="H63:H65"/>
+    <mergeCell ref="H66:H68"/>
+    <mergeCell ref="H69:H71"/>
+    <mergeCell ref="A83:A84"/>
+    <mergeCell ref="B83:B84"/>
+    <mergeCell ref="F83:F84"/>
+    <mergeCell ref="G83:G84"/>
+    <mergeCell ref="A57:A59"/>
+    <mergeCell ref="B57:B59"/>
+    <mergeCell ref="F57:F59"/>
+    <mergeCell ref="G57:G59"/>
+    <mergeCell ref="A69:A71"/>
+    <mergeCell ref="B69:B71"/>
+    <mergeCell ref="A72:A74"/>
+    <mergeCell ref="B72:B74"/>
+    <mergeCell ref="F69:F71"/>
+    <mergeCell ref="G69:G71"/>
+    <mergeCell ref="F72:F74"/>
+    <mergeCell ref="G72:G74"/>
+    <mergeCell ref="B63:B65"/>
+    <mergeCell ref="F63:F65"/>
+    <mergeCell ref="G63:G65"/>
+    <mergeCell ref="A66:A68"/>
+    <mergeCell ref="B66:B68"/>
+    <mergeCell ref="G66:G68"/>
+    <mergeCell ref="A75:A77"/>
+    <mergeCell ref="F60:F62"/>
+    <mergeCell ref="B75:B77"/>
+    <mergeCell ref="F75:F77"/>
+    <mergeCell ref="G75:G77"/>
+    <mergeCell ref="A33:A35"/>
+    <mergeCell ref="B33:B35"/>
+    <mergeCell ref="F33:F35"/>
+    <mergeCell ref="G33:G35"/>
+    <mergeCell ref="F42:F44"/>
+    <mergeCell ref="G42:G44"/>
+    <mergeCell ref="G48:G50"/>
+    <mergeCell ref="F66:F68"/>
+    <mergeCell ref="A51:A53"/>
+    <mergeCell ref="B51:B53"/>
+    <mergeCell ref="F51:F53"/>
+    <mergeCell ref="G51:G53"/>
+    <mergeCell ref="A54:A56"/>
+    <mergeCell ref="B54:B56"/>
+    <mergeCell ref="F54:F56"/>
+    <mergeCell ref="G54:G56"/>
+    <mergeCell ref="A60:A62"/>
+    <mergeCell ref="G27:G29"/>
+    <mergeCell ref="G60:G62"/>
+    <mergeCell ref="A63:A65"/>
+    <mergeCell ref="B42:B44"/>
+    <mergeCell ref="A42:A44"/>
+    <mergeCell ref="A39:A41"/>
+    <mergeCell ref="B39:B41"/>
+    <mergeCell ref="F39:F41"/>
+    <mergeCell ref="G39:G41"/>
+    <mergeCell ref="B60:B62"/>
+    <mergeCell ref="A36:A38"/>
+    <mergeCell ref="B36:B38"/>
+    <mergeCell ref="F45:F47"/>
+    <mergeCell ref="G45:G47"/>
+    <mergeCell ref="G88:G89"/>
+    <mergeCell ref="A90:A91"/>
+    <mergeCell ref="B90:B91"/>
+    <mergeCell ref="F90:F91"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B9:B11"/>
+    <mergeCell ref="A9:A11"/>
+    <mergeCell ref="F9:F11"/>
+    <mergeCell ref="G9:G11"/>
+    <mergeCell ref="A48:A50"/>
+    <mergeCell ref="B48:B50"/>
+    <mergeCell ref="F48:F50"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="B15:B17"/>
+    <mergeCell ref="F15:F17"/>
+    <mergeCell ref="G15:G17"/>
+    <mergeCell ref="A18:A20"/>
+    <mergeCell ref="A21:A23"/>
+    <mergeCell ref="B21:B23"/>
+    <mergeCell ref="F21:F23"/>
+    <mergeCell ref="G21:G23"/>
+    <mergeCell ref="A27:A29"/>
+    <mergeCell ref="B27:B29"/>
+    <mergeCell ref="F27:F29"/>
+    <mergeCell ref="G90:G91"/>
+    <mergeCell ref="A45:A47"/>
+    <mergeCell ref="B45:B47"/>
+    <mergeCell ref="F36:F38"/>
+    <mergeCell ref="G36:G38"/>
+    <mergeCell ref="A30:A32"/>
+    <mergeCell ref="B30:B32"/>
+    <mergeCell ref="F30:F32"/>
+    <mergeCell ref="G30:G32"/>
+    <mergeCell ref="A78:A80"/>
+    <mergeCell ref="B78:B80"/>
+    <mergeCell ref="F78:F80"/>
+    <mergeCell ref="G78:G80"/>
+    <mergeCell ref="A81:A82"/>
+    <mergeCell ref="B81:B82"/>
+    <mergeCell ref="F81:F82"/>
+    <mergeCell ref="G81:G82"/>
+    <mergeCell ref="A85:A87"/>
+    <mergeCell ref="B85:B87"/>
+    <mergeCell ref="F85:F87"/>
+    <mergeCell ref="G85:G87"/>
+    <mergeCell ref="A88:A89"/>
+    <mergeCell ref="B88:B89"/>
+    <mergeCell ref="F88:F89"/>
+    <mergeCell ref="F12:F14"/>
+    <mergeCell ref="G12:G14"/>
+    <mergeCell ref="B12:B14"/>
+    <mergeCell ref="A12:A14"/>
+    <mergeCell ref="B24:B26"/>
+    <mergeCell ref="A24:A26"/>
+    <mergeCell ref="F24:F26"/>
+    <mergeCell ref="G24:G26"/>
+    <mergeCell ref="B18:B20"/>
+    <mergeCell ref="F18:F20"/>
+    <mergeCell ref="G18:G20"/>
+    <mergeCell ref="A104:A106"/>
+    <mergeCell ref="B104:B106"/>
+    <mergeCell ref="F104:F106"/>
+    <mergeCell ref="G104:G106"/>
+    <mergeCell ref="A107:A109"/>
+    <mergeCell ref="B107:B109"/>
+    <mergeCell ref="F107:F109"/>
+    <mergeCell ref="G107:G109"/>
+    <mergeCell ref="A92:A94"/>
+    <mergeCell ref="B92:B94"/>
+    <mergeCell ref="F92:F94"/>
+    <mergeCell ref="G92:G94"/>
+    <mergeCell ref="A101:A103"/>
+    <mergeCell ref="B101:B103"/>
+    <mergeCell ref="F101:F103"/>
+    <mergeCell ref="G101:G103"/>
+    <mergeCell ref="G95:G97"/>
+    <mergeCell ref="A95:A97"/>
+    <mergeCell ref="B95:B97"/>
+    <mergeCell ref="F95:F97"/>
     <mergeCell ref="A98:A100"/>
     <mergeCell ref="B98:B100"/>
     <mergeCell ref="F98:F100"/>
@@ -3412,186 +3592,6 @@
     <mergeCell ref="F119:F121"/>
     <mergeCell ref="G119:G121"/>
     <mergeCell ref="G110:G112"/>
-    <mergeCell ref="A104:A106"/>
-    <mergeCell ref="B104:B106"/>
-    <mergeCell ref="F104:F106"/>
-    <mergeCell ref="G104:G106"/>
-    <mergeCell ref="A107:A109"/>
-    <mergeCell ref="B107:B109"/>
-    <mergeCell ref="F107:F109"/>
-    <mergeCell ref="G107:G109"/>
-    <mergeCell ref="A92:A94"/>
-    <mergeCell ref="B92:B94"/>
-    <mergeCell ref="F92:F94"/>
-    <mergeCell ref="G92:G94"/>
-    <mergeCell ref="F12:F14"/>
-    <mergeCell ref="G12:G14"/>
-    <mergeCell ref="B12:B14"/>
-    <mergeCell ref="A12:A14"/>
-    <mergeCell ref="B24:B26"/>
-    <mergeCell ref="A24:A26"/>
-    <mergeCell ref="F24:F26"/>
-    <mergeCell ref="G24:G26"/>
-    <mergeCell ref="B18:B20"/>
-    <mergeCell ref="F18:F20"/>
-    <mergeCell ref="G18:G20"/>
-    <mergeCell ref="G90:G91"/>
-    <mergeCell ref="A45:A47"/>
-    <mergeCell ref="B45:B47"/>
-    <mergeCell ref="F36:F38"/>
-    <mergeCell ref="G36:G38"/>
-    <mergeCell ref="A30:A32"/>
-    <mergeCell ref="B30:B32"/>
-    <mergeCell ref="F30:F32"/>
-    <mergeCell ref="G30:G32"/>
-    <mergeCell ref="A101:A103"/>
-    <mergeCell ref="B101:B103"/>
-    <mergeCell ref="F101:F103"/>
-    <mergeCell ref="G101:G103"/>
-    <mergeCell ref="A78:A80"/>
-    <mergeCell ref="B78:B80"/>
-    <mergeCell ref="F78:F80"/>
-    <mergeCell ref="G78:G80"/>
-    <mergeCell ref="A81:A82"/>
-    <mergeCell ref="B81:B82"/>
-    <mergeCell ref="F81:F82"/>
-    <mergeCell ref="G81:G82"/>
-    <mergeCell ref="A85:A87"/>
-    <mergeCell ref="B85:B87"/>
-    <mergeCell ref="F85:F87"/>
-    <mergeCell ref="G85:G87"/>
-    <mergeCell ref="G95:G97"/>
-    <mergeCell ref="A88:A89"/>
-    <mergeCell ref="B88:B89"/>
-    <mergeCell ref="F88:F89"/>
-    <mergeCell ref="G88:G89"/>
-    <mergeCell ref="A90:A91"/>
-    <mergeCell ref="B90:B91"/>
-    <mergeCell ref="F90:F91"/>
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B9:B11"/>
-    <mergeCell ref="A9:A11"/>
-    <mergeCell ref="F9:F11"/>
-    <mergeCell ref="G9:G11"/>
-    <mergeCell ref="A95:A97"/>
-    <mergeCell ref="B95:B97"/>
-    <mergeCell ref="F95:F97"/>
-    <mergeCell ref="A48:A50"/>
-    <mergeCell ref="B48:B50"/>
-    <mergeCell ref="F48:F50"/>
-    <mergeCell ref="A15:A17"/>
-    <mergeCell ref="B15:B17"/>
-    <mergeCell ref="F15:F17"/>
-    <mergeCell ref="G15:G17"/>
-    <mergeCell ref="A18:A20"/>
-    <mergeCell ref="A21:A23"/>
-    <mergeCell ref="B21:B23"/>
-    <mergeCell ref="F21:F23"/>
-    <mergeCell ref="G21:G23"/>
-    <mergeCell ref="A27:A29"/>
-    <mergeCell ref="B27:B29"/>
-    <mergeCell ref="F27:F29"/>
-    <mergeCell ref="G27:G29"/>
-    <mergeCell ref="G60:G62"/>
-    <mergeCell ref="A63:A65"/>
-    <mergeCell ref="B42:B44"/>
-    <mergeCell ref="A42:A44"/>
-    <mergeCell ref="A39:A41"/>
-    <mergeCell ref="B39:B41"/>
-    <mergeCell ref="F39:F41"/>
-    <mergeCell ref="G39:G41"/>
-    <mergeCell ref="B60:B62"/>
-    <mergeCell ref="A36:A38"/>
-    <mergeCell ref="B36:B38"/>
-    <mergeCell ref="F45:F47"/>
-    <mergeCell ref="G45:G47"/>
-    <mergeCell ref="B75:B77"/>
-    <mergeCell ref="F75:F77"/>
-    <mergeCell ref="G75:G77"/>
-    <mergeCell ref="A33:A35"/>
-    <mergeCell ref="B33:B35"/>
-    <mergeCell ref="F33:F35"/>
-    <mergeCell ref="G33:G35"/>
-    <mergeCell ref="F42:F44"/>
-    <mergeCell ref="G42:G44"/>
-    <mergeCell ref="G48:G50"/>
-    <mergeCell ref="F66:F68"/>
-    <mergeCell ref="A51:A53"/>
-    <mergeCell ref="B51:B53"/>
-    <mergeCell ref="F51:F53"/>
-    <mergeCell ref="G51:G53"/>
-    <mergeCell ref="A54:A56"/>
-    <mergeCell ref="B54:B56"/>
-    <mergeCell ref="F54:F56"/>
-    <mergeCell ref="G54:G56"/>
-    <mergeCell ref="A60:A62"/>
-    <mergeCell ref="A83:A84"/>
-    <mergeCell ref="B83:B84"/>
-    <mergeCell ref="F83:F84"/>
-    <mergeCell ref="G83:G84"/>
-    <mergeCell ref="A57:A59"/>
-    <mergeCell ref="B57:B59"/>
-    <mergeCell ref="F57:F59"/>
-    <mergeCell ref="G57:G59"/>
-    <mergeCell ref="A69:A71"/>
-    <mergeCell ref="B69:B71"/>
-    <mergeCell ref="A72:A74"/>
-    <mergeCell ref="B72:B74"/>
-    <mergeCell ref="F69:F71"/>
-    <mergeCell ref="G69:G71"/>
-    <mergeCell ref="F72:F74"/>
-    <mergeCell ref="G72:G74"/>
-    <mergeCell ref="B63:B65"/>
-    <mergeCell ref="F63:F65"/>
-    <mergeCell ref="G63:G65"/>
-    <mergeCell ref="A66:A68"/>
-    <mergeCell ref="B66:B68"/>
-    <mergeCell ref="G66:G68"/>
-    <mergeCell ref="A75:A77"/>
-    <mergeCell ref="F60:F62"/>
-    <mergeCell ref="C116:C118"/>
-    <mergeCell ref="D116:D118"/>
-    <mergeCell ref="E116:E118"/>
-    <mergeCell ref="H9:H11"/>
-    <mergeCell ref="H12:H14"/>
-    <mergeCell ref="H15:H17"/>
-    <mergeCell ref="H18:H20"/>
-    <mergeCell ref="H21:H23"/>
-    <mergeCell ref="H24:H26"/>
-    <mergeCell ref="H27:H29"/>
-    <mergeCell ref="H30:H32"/>
-    <mergeCell ref="H33:H35"/>
-    <mergeCell ref="H36:H38"/>
-    <mergeCell ref="H39:H41"/>
-    <mergeCell ref="H42:H44"/>
-    <mergeCell ref="H45:H47"/>
-    <mergeCell ref="H48:H50"/>
-    <mergeCell ref="H51:H53"/>
-    <mergeCell ref="H54:H56"/>
-    <mergeCell ref="H57:H59"/>
-    <mergeCell ref="H60:H62"/>
-    <mergeCell ref="H63:H65"/>
-    <mergeCell ref="H66:H68"/>
-    <mergeCell ref="H69:H71"/>
-    <mergeCell ref="H72:H74"/>
-    <mergeCell ref="H75:H77"/>
-    <mergeCell ref="H78:H80"/>
-    <mergeCell ref="H83:H84"/>
-    <mergeCell ref="H81:H82"/>
-    <mergeCell ref="H85:H87"/>
-    <mergeCell ref="H88:H89"/>
-    <mergeCell ref="H90:H91"/>
-    <mergeCell ref="H92:H94"/>
-    <mergeCell ref="H122:H124"/>
-    <mergeCell ref="H95:H97"/>
-    <mergeCell ref="H98:H100"/>
-    <mergeCell ref="H101:H103"/>
-    <mergeCell ref="H104:H106"/>
-    <mergeCell ref="H107:H109"/>
-    <mergeCell ref="H110:H112"/>
-    <mergeCell ref="H113:H115"/>
-    <mergeCell ref="H116:H118"/>
-    <mergeCell ref="H119:H121"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="3" orientation="landscape" r:id="rId1"/>

</xml_diff>